<commit_message>
Completed Day5 work of Power Functions & Visual Formatting
</commit_message>
<xml_diff>
--- a/Day3/Lookup Functions & Data Quality.xlsx
+++ b/Day3/Lookup Functions & Data Quality.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\Mine\Data Analytics Practises\Day3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99699F20-0C56-4CEC-9E93-C2A6F7DA97FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B16BED6-8935-4798-9C80-16FBB50F91B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,30 +32,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="66">
   <si>
     <t>ProductID</t>
   </si>
@@ -211,9 +189,6 @@
   </si>
   <si>
     <t>IFERROR:</t>
-  </si>
-  <si>
-    <t>Pencil</t>
   </si>
   <si>
     <t>PRICE</t>
@@ -330,7 +305,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -348,6 +333,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -691,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -828,7 +823,7 @@
         <v>179.93</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -859,8 +854,8 @@
       <c r="I5" s="2">
         <v>159.55000000000001</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>4</v>
+      <c r="K5" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -868,7 +863,7 @@
         <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C6" s="2">
         <v>442</v>
@@ -892,9 +887,8 @@
         <v>2.02</v>
       </c>
       <c r="J6" s="4"/>
-      <c r="K6" s="2" t="str">
-        <f>IFERROR(VLOOKUP(K4,B1:I15,4,FALSE),"NO ITEM")</f>
-        <v>NO ITEM</v>
+      <c r="K6" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -925,8 +919,8 @@
       <c r="I7" s="2">
         <v>116.17</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>6</v>
+      <c r="K7" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
@@ -957,9 +951,8 @@
       <c r="I8" s="2">
         <v>157.27000000000001</v>
       </c>
-      <c r="K8" s="2" t="str" cm="1">
-        <f t="array" ref="K8">IFERROR(_xlfn.XLOOKUP(K4,A1,E1:F15),"NO ITEM")</f>
-        <v>NO ITEM</v>
+      <c r="K8" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -1112,7 +1105,7 @@
         <v>21</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C14" s="2">
         <v>437</v>
@@ -1141,7 +1134,7 @@
         <v>22</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C15" s="2">
         <v>301</v>
@@ -1180,7 +1173,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="K21" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
@@ -1206,7 +1199,7 @@
         <v>45</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
@@ -1259,7 +1252,7 @@
         <v>20</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
@@ -1297,24 +1290,24 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="D30" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="F30" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B31" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C31" s="2" t="str">
         <f>UPPER(F31)</f>
@@ -1335,7 +1328,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B32" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C32" s="2" t="str">
         <f t="shared" ref="C32:C34" si="0">UPPER(F32)</f>
@@ -1356,7 +1349,7 @@
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B33" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C33" s="2" t="str">
         <f t="shared" si="0"/>
@@ -1377,7 +1370,7 @@
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B34" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C34" s="2" t="str">
         <f t="shared" si="0"/>
@@ -1398,7 +1391,7 @@
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.3">
       <c r="E40" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.3">
@@ -1461,155 +1454,65 @@
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B44" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D44" s="2">
-        <v>15</v>
+        <v>442</v>
       </c>
       <c r="E44" s="2">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H44" s="2">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J44" s="2">
-        <v>179.93</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B45" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D45" s="2">
-        <v>35</v>
+        <v>396</v>
       </c>
       <c r="E45" s="2">
-        <v>56</v>
+        <v>84</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H45" s="2">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J45" s="2">
-        <v>159.55000000000001</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B46" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D46" s="2">
-        <v>442</v>
-      </c>
-      <c r="E46" s="2">
-        <v>64</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H46" s="2">
-        <v>8</v>
-      </c>
-      <c r="I46" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J46" s="2">
-        <v>2.02</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B47" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D47" s="2">
-        <v>396</v>
-      </c>
-      <c r="E47" s="2">
-        <v>84</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H47" s="2">
-        <v>17</v>
-      </c>
-      <c r="I47" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J47" s="2">
         <v>147.57</v>
-      </c>
-    </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B48" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D48" s="2">
-        <v>163</v>
-      </c>
-      <c r="E48" s="2">
-        <v>44</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H48" s="2">
-        <v>17</v>
-      </c>
-      <c r="I48" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="J48" s="2">
-        <v>155.35</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J1:J15">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B42:E48">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>